<commit_message>
corrección puntual de las historias de usuario.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Documentación/Historias de Usuario y criterios de aceptación SIGET.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Documentación/Historias de Usuario y criterios de aceptación SIGET.xlsx
@@ -775,22 +775,22 @@
     <t xml:space="preserve">Con la finalidad de asignar responsables, atender las solicitudes y mantener actualizado su estado.</t>
   </si>
   <si>
-    <t xml:space="preserve">Asignación o reasignación de ticket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso que exista un ticket pendiente de asignación o que requiera cambio de responsable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuando el Administrador del sistema asigna o reasigna el ticket a un Técnico de soporte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema registra al Técnico responsable y mantiene trazabilidad de la asignación o reasignación</t>
+    <t xml:space="preserve">Asignación administrativa y toma de tickets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso que exista un ticket activo sin Técnico responsable, o que se requiera asignar o reasignar un ticket activo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuando el Administrador asigna o reasigna el ticket, o un Técnico toma para sí un ticket sin responsable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema registra al responsable y audita la operación. Solo el Administrador puede asignar a otro Técnico o reasignar. Ante tomas simultáneas solo una confirma, sin sobrescribir al responsable.</t>
   </si>
   <si>
     <t xml:space="preserve">Atención y cambio de estado</t>
   </si>
   <si>
-    <t xml:space="preserve">En caso que el técnico tenga un ticket asignado</t>
+    <t xml:space="preserve">En caso que el Técnico sea el responsable asignado del ticket</t>
   </si>
   <si>
     <t xml:space="preserve">Cuando el Técnico registra la atención realizada o modifica el estado del ticket</t>
@@ -811,16 +811,16 @@
     <t xml:space="preserve">El sistema informa que el ticket no existe</t>
   </si>
   <si>
-    <t xml:space="preserve">Ticket cerrado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso que el ticket se encuentre cerrado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuando el técnico intenta modificarlo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema informa que el ticket se encuentra cerrado y no permite modificarlo</t>
+    <t xml:space="preserve">Ticket cerrado o toma no permitida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En caso que el ticket esté cerrado, o que al intentar tomarlo esté resuelto o asignado a otro Técnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuando el Técnico intenta modificar el ticket cerrado o tomar un ticket no disponible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema rechaza la operación sin modificar el ticket, su estado ni su responsable.</t>
   </si>
   <si>
     <t>E5-H15</t>
@@ -1816,38 +1816,38 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="none"/>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -1856,42 +1856,42 @@
       <right style="none"/>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="none"/>
       <bottom style="none"/>
@@ -5164,7 +5164,7 @@
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" ht="15">
+    <row r="72" ht="80.25" customHeight="1">
       <c r="A72" s="1"/>
       <c r="B72" s="14"/>
       <c r="C72" s="14"/>
@@ -5202,7 +5202,7 @@
       <c r="Y72" s="1"/>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" ht="15">
+    <row r="73" ht="63.75" customHeight="1">
       <c r="A73" s="1"/>
       <c r="B73" s="14"/>
       <c r="C73" s="14"/>
@@ -5240,7 +5240,7 @@
       <c r="Y73" s="1"/>
       <c r="Z73" s="1"/>
     </row>
-    <row r="74" ht="15">
+    <row r="74" ht="84" customHeight="1">
       <c r="A74" s="1"/>
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>

</xml_diff>